<commit_message>
MAJ suite aux retours 8662296a57d1e78356f76f28930bd9e84a0add3c
</commit_message>
<xml_diff>
--- a/htr-FHIR/ig/StructureDefinition-fr-human-name-document.xlsx
+++ b/htr-FHIR/ig/StructureDefinition-fr-human-name-document.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-23T09:31:53+00:00</t>
+    <t>2025-04-24T14:52:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Ce profil représente le nom du professionnel de santé.</t>
+    <t>Ce profil correspond au type de données HumanName utilisé dans le document.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -1783,7 +1783,7 @@
         <v>77</v>
       </c>
       <c r="G9" t="s" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H9" t="s" s="2">
         <v>76</v>

</xml_diff>